<commit_message>
Extend mass import for centerId
</commit_message>
<xml_diff>
--- a/shanoir-uploader/src/test/resources/template_pacs_import.xlsx
+++ b/shanoir-uploader/src/test/resources/template_pacs_import.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="22">
   <si>
     <t xml:space="preserve">DICOM_QUERY_LEVEL</t>
   </si>
@@ -65,6 +65,9 @@
   </si>
   <si>
     <t xml:space="preserve">SHANOIR_STUDY_CARD_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SHANOIR_CENTER_ID</t>
   </si>
   <si>
     <t xml:space="preserve">SHANOIR_SUBJECT_NAME</t>
@@ -410,7 +413,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Q3"/>
+  <dimension ref="A1:R3"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="21.88"/>
@@ -426,8 +429,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="11" style="2" width="34.97"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="34.97"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="2" width="34.97"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="2" width="25.35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="2" width="26.32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="16" style="2" width="25.35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="2" width="26.32"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -482,35 +485,38 @@
       <c r="Q1" s="7" t="s">
         <v>16</v>
       </c>
+      <c r="R1" s="7" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I2" s="8"/>
       <c r="N2" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I3" s="8"/>
       <c r="N3" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>